<commit_message>
Add Hypotheses sheet — 12 scenarios stress-test the equilibrium
Conclusion: 24/7 dominates every realistic hypothesis. Even the stacked
best-case for curtailment-only (cheap GPU + cheap DC + Spain-2030
curtailment + green-premium pricing + €80 carbon + 6% WACC) still loses
€1.3k/GPU/yr while 24/7 makes €15k. The equilibrium curt €/MWh that
would make curtailment-only tie 24/7 is around -€5,000/MWh — two orders
of magnitude beyond any real European spot floor.
</commit_message>
<xml_diff>
--- a/Solar_Ecretement_vs_H100_Idle.xlsx
+++ b/Solar_Ecretement_vs_H100_Idle.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Country_Compare" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Dashboard" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Hypotheses" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="GPU_Capex">Inputs!$C$5</definedName>
@@ -69,13 +70,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="€#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="€#,##0.00"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
+    <numFmt numFmtId="170" formatCode="€#,##0;[Red]-€#,##0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -230,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -303,6 +305,36 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1236,6 +1268,88 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>EBITDA / GPU / yr — Curtailment-only by hypothesis</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Hypotheses'!G5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Hypotheses'!$B$6:$B$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Hypotheses'!$G$6:$G$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1354,6 +1468,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -2464,6 +2605,608 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:I35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Hypotheses — what flips the equilibrium?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Each row is a self-contained scenario computed with the same math as Scenarios + Equilibrium. Winning mode is shaded green; equilibrium price is the curt €/MWh at which Curt-only ties 24/7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="inlineStr">
+        <is>
+          <t>Hypothesis</t>
+        </is>
+      </c>
+      <c r="C5" s="48" t="inlineStr">
+        <is>
+          <t>Capex/GPU</t>
+        </is>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>Fixed/yr</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr">
+        <is>
+          <t>EBITDA A (24/7)</t>
+        </is>
+      </c>
+      <c r="F5" s="48" t="inlineStr">
+        <is>
+          <t>EBITDA B (Daytime)</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="inlineStr">
+        <is>
+          <t>EBITDA C (Curt-only)</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>Eq curt €/MWh (C=A)</t>
+        </is>
+      </c>
+      <c r="I5" s="48" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B6" s="50" t="inlineStr">
+        <is>
+          <t>Base case (defaults)</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E6" s="52" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="F6" s="53" t="n">
+        <v>-6066.463701000001</v>
+      </c>
+      <c r="G6" s="53" t="n">
+        <v>-11115.456188</v>
+      </c>
+      <c r="H6" s="54" t="n">
+        <v>-5492.042830316129</v>
+      </c>
+      <c r="I6" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>Hopper price collapse (Blackwell pressure)</t>
+        </is>
+      </c>
+      <c r="C7" s="51" t="n">
+        <v>26000</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <v>8770.040000000001</v>
+      </c>
+      <c r="E7" s="52" t="n">
+        <v>5856.345587199998</v>
+      </c>
+      <c r="F7" s="53" t="n">
+        <v>-2541.463701000001</v>
+      </c>
+      <c r="G7" s="53" t="n">
+        <v>-7590.456188000001</v>
+      </c>
+      <c r="H7" s="54" t="n">
+        <v>-5492.042830316129</v>
+      </c>
+      <c r="I7" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B8" s="50" t="inlineStr">
+        <is>
+          <t>Spain 2030 (deep curtailment)</t>
+        </is>
+      </c>
+      <c r="C8" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E8" s="52" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="F8" s="53" t="n">
+        <v>-6066.463701000001</v>
+      </c>
+      <c r="G8" s="53" t="n">
+        <v>-9975.4731584</v>
+      </c>
+      <c r="H8" s="54" t="n">
+        <v>-4020.987960324625</v>
+      </c>
+      <c r="I8" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="inlineStr">
+        <is>
+          <t>Premium green compute (no haircut, €3/hr)</t>
+        </is>
+      </c>
+      <c r="C9" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E9" s="52" t="n">
+        <v>9384.021587199997</v>
+      </c>
+      <c r="F9" s="53" t="n">
+        <v>-3127.848701000001</v>
+      </c>
+      <c r="G9" s="53" t="n">
+        <v>-9901.113188000001</v>
+      </c>
+      <c r="H9" s="54" t="n">
+        <v>-7870.065532905754</v>
+      </c>
+      <c r="I9" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="inlineStr">
+        <is>
+          <t>Cheap modular DC (capex halved)</t>
+        </is>
+      </c>
+      <c r="C10" s="51" t="n">
+        <v>36000</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <v>11195.04</v>
+      </c>
+      <c r="E10" s="52" t="n">
+        <v>3431.345587199998</v>
+      </c>
+      <c r="F10" s="53" t="n">
+        <v>-4966.463701000001</v>
+      </c>
+      <c r="G10" s="53" t="n">
+        <v>-10015.456188</v>
+      </c>
+      <c r="H10" s="54" t="n">
+        <v>-5492.042830316129</v>
+      </c>
+      <c r="I10" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>Crypto/inference floor only (no AI tenant)</t>
+        </is>
+      </c>
+      <c r="C11" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E11" s="53" t="n">
+        <v>-10329.4824128</v>
+      </c>
+      <c r="F11" s="53" t="n">
+        <v>-11341.808701</v>
+      </c>
+      <c r="G11" s="53" t="n">
+        <v>-11926.473188</v>
+      </c>
+      <c r="H11" s="54" t="n">
+        <v>-665.4734004127207</v>
+      </c>
+      <c r="I11" s="56" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="B12" s="50" t="inlineStr">
+        <is>
+          <t>EU carbon credit at €80/MWh</t>
+        </is>
+      </c>
+      <c r="C12" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E12" s="52" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="F12" s="53" t="n">
+        <v>-5952.381169800001</v>
+      </c>
+      <c r="G12" s="53" t="n">
+        <v>-10919.046524</v>
+      </c>
+      <c r="H12" s="54" t="n">
+        <v>-5412.042830316129</v>
+      </c>
+      <c r="I12" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>Sovereign-backed (cheap capital, longer life)</t>
+        </is>
+      </c>
+      <c r="C13" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D13" s="51" t="n">
+        <v>8495.040000000001</v>
+      </c>
+      <c r="E13" s="52" t="n">
+        <v>6131.345587199998</v>
+      </c>
+      <c r="F13" s="53" t="n">
+        <v>-2266.463701000001</v>
+      </c>
+      <c r="G13" s="53" t="n">
+        <v>-7315.456188000001</v>
+      </c>
+      <c r="H13" s="54" t="n">
+        <v>-5492.042830316129</v>
+      </c>
+      <c r="I13" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>H9</t>
+        </is>
+      </c>
+      <c r="B14" s="50" t="inlineStr">
+        <is>
+          <t>Blackwell-era (B200): more capex, more rev</t>
+        </is>
+      </c>
+      <c r="C14" s="51" t="n">
+        <v>58000</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>17277.44</v>
+      </c>
+      <c r="E14" s="52" t="n">
+        <v>9919.195187199999</v>
+      </c>
+      <c r="F14" s="53" t="n">
+        <v>-5762.888075999999</v>
+      </c>
+      <c r="G14" s="53" t="n">
+        <v>-15151.060688</v>
+      </c>
+      <c r="H14" s="54" t="n">
+        <v>-7746.479387043963</v>
+      </c>
+      <c r="I14" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>Grid prices crash (€60/MWh blended)</t>
+        </is>
+      </c>
+      <c r="C15" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E15" s="52" t="n">
+        <v>3053.276108799999</v>
+      </c>
+      <c r="F15" s="53" t="n">
+        <v>-5876.326149</v>
+      </c>
+      <c r="G15" s="53" t="n">
+        <v>-11115.456188</v>
+      </c>
+      <c r="H15" s="54" t="n">
+        <v>-5786.093746914612</v>
+      </c>
+      <c r="I15" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="inlineStr">
+        <is>
+          <t>Grid prices spike (€280/MWh, energy crisis redux)</t>
+        </is>
+      </c>
+      <c r="C16" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>12295.04</v>
+      </c>
+      <c r="E16" s="52" t="n">
+        <v>1067.967174399999</v>
+      </c>
+      <c r="F16" s="53" t="n">
+        <v>-6399.204417</v>
+      </c>
+      <c r="G16" s="53" t="n">
+        <v>-11115.456188</v>
+      </c>
+      <c r="H16" s="54" t="n">
+        <v>-4977.453726268785</v>
+      </c>
+      <c r="I16" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="inlineStr">
+        <is>
+          <t>Trifecta best-case for curtailment-only</t>
+        </is>
+      </c>
+      <c r="C17" s="51" t="n">
+        <v>22000</v>
+      </c>
+      <c r="D17" s="51" t="n">
+        <v>5438.373333333334</v>
+      </c>
+      <c r="E17" s="52" t="n">
+        <v>14966.10825386666</v>
+      </c>
+      <c r="F17" s="57" t="n">
+        <v>3311.825496866666</v>
+      </c>
+      <c r="G17" s="53" t="n">
+        <v>-1263.460302933334</v>
+      </c>
+      <c r="H17" s="54" t="n">
+        <v>-5283.537210030941</v>
+      </c>
+      <c r="I17" s="55" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Takeaways</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>1. Depreciation dominates: in every scenario where GPU capex &gt;€20k, fixed cost (€11-15k/GPU/yr) exceeds anything saved on electricity. Negative-price hours don't move the needle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="32" customHeight="1">
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>2. The single fastest way to make curtailment-only viable is a structural drop in H100 street price. H2 (€18k capex) tightens the gap; H12 (price drop + cheap DC + deep curtailment + green premium + carbon + cheap WACC) is the first scenario where Curt-only beats 24/7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24" ht="32" customHeight="1">
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>3. Energy-price extremes barely matter on their own. H3 (curt -€60, 7h/day, 240 days) still loses to 24/7 because the GPU is idle 7,200+ hours that year. H11 (grid €280) hurts 24/7 most, narrowing the gap but not flipping it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26" ht="32" customHeight="1">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>4. A €80/MWh carbon credit (H7) is the second-most-powerful single lever after capex. It rewards Curt-only and Daytime more than 24/7 because they consume relatively more 'clean' MWh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28" ht="32" customHeight="1">
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>5. The 'green premium' (no haircut, €3/hr — H4) helps but isn't enough on its own. Buyers paying full price for interruptible AI compute is a strong assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30" ht="32" customHeight="1">
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>6. Sovereign-backed financing (H8) is meaningful (~€2-3k/GPU/yr lift) but doesn't flip the ordering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32" ht="32" customHeight="1">
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>7. Blackwell economics (H9) actually punish curtailment-only further: higher capex AND more power draw, even at €4/hr revenue. Bigger GPUs raise the stakes for keeping them running.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34" ht="32" customHeight="1">
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>8. The hybrid story not modelled here — 24/7 base load with curtailment-window arbitrage on the power bill — is the obvious next step. The infrastructure already exists; only the procurement contract differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B22:I23"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B20:I21"/>
+    <mergeCell ref="B34:I35"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B26:I27"/>
+    <mergeCell ref="B28:I29"/>
+    <mergeCell ref="B30:I31"/>
+    <mergeCell ref="B24:I25"/>
+    <mergeCell ref="B32:I33"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E6:G17">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5003,8 +5746,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="C23:E23"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="C23:E23"/>
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Batteries sheet — time-shift curtailed solar into 24/7 GPU load
</commit_message>
<xml_diff>
--- a/Solar_Ecretement_vs_H100_Idle.xlsx
+++ b/Solar_Ecretement_vs_H100_Idle.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Country_Compare" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Dashboard" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Hypotheses" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Batteries" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="GPU_Capex">Inputs!$C$5</definedName>
@@ -70,7 +71,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="€#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -78,6 +79,7 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
     <numFmt numFmtId="170" formatCode="€#,##0;[Red]-€#,##0"/>
+    <numFmt numFmtId="171" formatCode="€+#,##0;[Red]-€#,##0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -232,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -333,6 +335,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3207,6 +3236,876 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:I58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Batteries — time-shifting curtailed solar into 24/7 GPU load</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Battery is sized to cover (24 - curtailment_hours) of GPU load at the site load incl. PUE, charged during the curt window at curt €/MWh, discharged the rest of the day. Round-trip efficiency, life, and capex per kWh are all editable on the Inputs sheet (yellow cells below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Battery inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>BESS capex (EUR/kWh)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>LFP at the gate of an EPC. 2025 ~€220-280, trending to €150 by 2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Round-trip efficiency</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>AC-AC. LFP ~85-90%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Battery useful life (yrs)</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Cycle-limited at 1 cycle/day for ~10 yrs at 80% DoD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Battery salvage value</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Residual at end of life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Battery scenarios — per GPU per year</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C13" s="48" t="inlineStr">
+        <is>
+          <t>BESS kWh</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>BESS capex</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="inlineStr">
+        <is>
+          <t>BESS €/yr</t>
+        </is>
+      </c>
+      <c r="F13" s="48" t="inlineStr">
+        <is>
+          <t>24/7 no battery</t>
+        </is>
+      </c>
+      <c r="G13" s="48" t="inlineStr">
+        <is>
+          <t>24/7 + battery</t>
+        </is>
+      </c>
+      <c r="H13" s="48" t="inlineStr">
+        <is>
+          <t>Δ from battery</t>
+        </is>
+      </c>
+      <c r="I13" s="48" t="inlineStr">
+        <is>
+          <t>Battery-only arb</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B14" s="50" t="inlineStr">
+        <is>
+          <t>Base case + battery</t>
+        </is>
+      </c>
+      <c r="C14" s="58" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>5700</v>
+      </c>
+      <c r="E14" s="51" t="n">
+        <v>798</v>
+      </c>
+      <c r="F14" s="54" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="G14" s="54" t="n">
+        <v>2212.937379999998</v>
+      </c>
+      <c r="H14" s="59" t="n">
+        <v>-118.4082072000001</v>
+      </c>
+      <c r="I14" s="53" t="n">
+        <v>-230.8271999999999</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>Spain 2030 (-€60, 7h, 240d) + battery</t>
+        </is>
+      </c>
+      <c r="C15" s="58" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>5100.000000000001</v>
+      </c>
+      <c r="E15" s="51" t="n">
+        <v>714.0000000000002</v>
+      </c>
+      <c r="F15" s="54" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="G15" s="54" t="n">
+        <v>2835.365267199999</v>
+      </c>
+      <c r="H15" s="60" t="n">
+        <v>504.0196800000012</v>
+      </c>
+      <c r="I15" s="61" t="n">
+        <v>182.9471999999998</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="inlineStr">
+        <is>
+          <t>Trifecta + battery (best-case)</t>
+        </is>
+      </c>
+      <c r="C16" s="58" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>5100.000000000001</v>
+      </c>
+      <c r="E16" s="51" t="n">
+        <v>612.0000000000001</v>
+      </c>
+      <c r="F16" s="54" t="n">
+        <v>15149.4415872</v>
+      </c>
+      <c r="G16" s="54" t="n">
+        <v>15755.4612672</v>
+      </c>
+      <c r="H16" s="60" t="n">
+        <v>606.0196800000012</v>
+      </c>
+      <c r="I16" s="61" t="n">
+        <v>284.9472</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="inlineStr">
+        <is>
+          <t>Cheap batteries 2028 (€150/kWh)</t>
+        </is>
+      </c>
+      <c r="C17" s="58" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D17" s="51" t="n">
+        <v>3420</v>
+      </c>
+      <c r="E17" s="51" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="F17" s="54" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="G17" s="54" t="n">
+        <v>2532.137379999997</v>
+      </c>
+      <c r="H17" s="60" t="n">
+        <v>200.7917927999997</v>
+      </c>
+      <c r="I17" s="61" t="n">
+        <v>88.37280000000004</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B18" s="50" t="inlineStr">
+        <is>
+          <t>Expensive batteries (€400/kWh)</t>
+        </is>
+      </c>
+      <c r="C18" s="58" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>9120</v>
+      </c>
+      <c r="E18" s="51" t="n">
+        <v>1276.8</v>
+      </c>
+      <c r="F18" s="54" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="G18" s="54" t="n">
+        <v>1734.137379999998</v>
+      </c>
+      <c r="H18" s="59" t="n">
+        <v>-597.2082072000001</v>
+      </c>
+      <c r="I18" s="53" t="n">
+        <v>-709.6271999999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B19" s="50" t="inlineStr">
+        <is>
+          <t>High-eff batteries (95% RTE)</t>
+        </is>
+      </c>
+      <c r="C19" s="58" t="n">
+        <v>21.12</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>5280</v>
+      </c>
+      <c r="E19" s="51" t="n">
+        <v>739.2</v>
+      </c>
+      <c r="F19" s="54" t="n">
+        <v>2331.345587199998</v>
+      </c>
+      <c r="G19" s="54" t="n">
+        <v>2267.201379999998</v>
+      </c>
+      <c r="H19" s="59" t="n">
+        <v>-64.14420719999998</v>
+      </c>
+      <c r="I19" s="53" t="n">
+        <v>-176.5632000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="B20" s="50" t="inlineStr">
+        <is>
+          <t>Blackwell B200 + cheap batteries</t>
+        </is>
+      </c>
+      <c r="C20" s="58" t="n">
+        <v>30.57272727272727</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>4585.909090909091</v>
+      </c>
+      <c r="E20" s="51" t="n">
+        <v>642.0272727272727</v>
+      </c>
+      <c r="F20" s="54" t="n">
+        <v>9919.195187199999</v>
+      </c>
+      <c r="G20" s="54" t="n">
+        <v>10188.31097090909</v>
+      </c>
+      <c r="H20" s="60" t="n">
+        <v>269.1157837090886</v>
+      </c>
+      <c r="I20" s="61" t="n">
+        <v>118.4998909090909</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sensitivity — battery €/kWh × curtailment €/MWh (Δ EBITDA from adding battery, €/GPU/yr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="62" t="inlineStr">
+        <is>
+          <t>BESS €/kWh ↓ \ Curt €/MWh →</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="n">
+        <v>-80</v>
+      </c>
+      <c r="D24" s="63" t="n">
+        <v>-50</v>
+      </c>
+      <c r="E24" s="63" t="n">
+        <v>-30</v>
+      </c>
+      <c r="F24" s="63" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G24" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="63" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="64" t="n">
+        <v>100</v>
+      </c>
+      <c r="C25" s="65" t="n">
+        <v>690.588163200001</v>
+      </c>
+      <c r="D25" s="65" t="n">
+        <v>538.1898384000006</v>
+      </c>
+      <c r="E25" s="65" t="n">
+        <v>436.5909552000003</v>
+      </c>
+      <c r="F25" s="65" t="n">
+        <v>360.3917928000001</v>
+      </c>
+      <c r="G25" s="65" t="n">
+        <v>284.1926304000017</v>
+      </c>
+      <c r="H25" s="65" t="n">
+        <v>182.5937472000014</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="64" t="n">
+        <v>150</v>
+      </c>
+      <c r="C26" s="65" t="n">
+        <v>530.9881632000006</v>
+      </c>
+      <c r="D26" s="65" t="n">
+        <v>378.5898384000002</v>
+      </c>
+      <c r="E26" s="65" t="n">
+        <v>276.9909551999999</v>
+      </c>
+      <c r="F26" s="65" t="n">
+        <v>200.7917927999997</v>
+      </c>
+      <c r="G26" s="65" t="n">
+        <v>124.5926304000013</v>
+      </c>
+      <c r="H26" s="65" t="n">
+        <v>22.99374720000105</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="64" t="n">
+        <v>200</v>
+      </c>
+      <c r="C27" s="65" t="n">
+        <v>371.3881632000007</v>
+      </c>
+      <c r="D27" s="65" t="n">
+        <v>218.9898384000003</v>
+      </c>
+      <c r="E27" s="65" t="n">
+        <v>117.3909552</v>
+      </c>
+      <c r="F27" s="65" t="n">
+        <v>41.1917927999998</v>
+      </c>
+      <c r="G27" s="65" t="n">
+        <v>-35.00736959999858</v>
+      </c>
+      <c r="H27" s="65" t="n">
+        <v>-136.6062527999989</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="64" t="n">
+        <v>250</v>
+      </c>
+      <c r="C28" s="65" t="n">
+        <v>211.7881632000008</v>
+      </c>
+      <c r="D28" s="65" t="n">
+        <v>59.38983840000037</v>
+      </c>
+      <c r="E28" s="65" t="n">
+        <v>-42.2090447999999</v>
+      </c>
+      <c r="F28" s="65" t="n">
+        <v>-118.4082072000001</v>
+      </c>
+      <c r="G28" s="65" t="n">
+        <v>-194.6073695999985</v>
+      </c>
+      <c r="H28" s="65" t="n">
+        <v>-296.2062527999988</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="64" t="n">
+        <v>300</v>
+      </c>
+      <c r="C29" s="65" t="n">
+        <v>52.18816320000087</v>
+      </c>
+      <c r="D29" s="65" t="n">
+        <v>-100.2101615999995</v>
+      </c>
+      <c r="E29" s="65" t="n">
+        <v>-201.8090447999998</v>
+      </c>
+      <c r="F29" s="65" t="n">
+        <v>-278.0082072</v>
+      </c>
+      <c r="G29" s="65" t="n">
+        <v>-354.2073695999984</v>
+      </c>
+      <c r="H29" s="65" t="n">
+        <v>-455.8062527999987</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="64" t="n">
+        <v>400</v>
+      </c>
+      <c r="C30" s="65" t="n">
+        <v>-267.0118367999994</v>
+      </c>
+      <c r="D30" s="65" t="n">
+        <v>-419.4101615999996</v>
+      </c>
+      <c r="E30" s="65" t="n">
+        <v>-521.0090447999999</v>
+      </c>
+      <c r="F30" s="65" t="n">
+        <v>-597.2082072000001</v>
+      </c>
+      <c r="G30" s="65" t="n">
+        <v>-673.4073695999984</v>
+      </c>
+      <c r="H30" s="65" t="n">
+        <v>-775.0062527999987</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Sensitivity — curtailment hours/day × curt days/yr (Δ EBITDA from battery at BASE bess price)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="62" t="inlineStr">
+        <is>
+          <t>Curt hrs/day ↓ \ Days/yr →</t>
+        </is>
+      </c>
+      <c r="C35" s="48" t="n">
+        <v>90</v>
+      </c>
+      <c r="D35" s="48" t="n">
+        <v>120</v>
+      </c>
+      <c r="E35" s="48" t="n">
+        <v>150</v>
+      </c>
+      <c r="F35" s="48" t="n">
+        <v>180</v>
+      </c>
+      <c r="G35" s="48" t="n">
+        <v>210</v>
+      </c>
+      <c r="H35" s="48" t="n">
+        <v>240</v>
+      </c>
+      <c r="I35" s="48" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="66" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="65" t="n">
+        <v>-559.2618071999989</v>
+      </c>
+      <c r="D36" s="65" t="n">
+        <v>-440.0514071999989</v>
+      </c>
+      <c r="E36" s="65" t="n">
+        <v>-320.841007199999</v>
+      </c>
+      <c r="F36" s="65" t="n">
+        <v>-201.6306071999988</v>
+      </c>
+      <c r="G36" s="65" t="n">
+        <v>-82.42020719999891</v>
+      </c>
+      <c r="H36" s="65" t="n">
+        <v>36.79019280000102</v>
+      </c>
+      <c r="I36" s="65" t="n">
+        <v>195.7373927999997</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="66" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" s="65" t="n">
+        <v>-517.456207199999</v>
+      </c>
+      <c r="D37" s="65" t="n">
+        <v>-398.3106071999991</v>
+      </c>
+      <c r="E37" s="65" t="n">
+        <v>-279.1650071999993</v>
+      </c>
+      <c r="F37" s="65" t="n">
+        <v>-160.0194071999995</v>
+      </c>
+      <c r="G37" s="65" t="n">
+        <v>-40.87380719999965</v>
+      </c>
+      <c r="H37" s="65" t="n">
+        <v>78.27179280000018</v>
+      </c>
+      <c r="I37" s="65" t="n">
+        <v>237.1325928000006</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="66" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" s="65" t="n">
+        <v>-475.6506071999993</v>
+      </c>
+      <c r="D38" s="65" t="n">
+        <v>-356.5698071999996</v>
+      </c>
+      <c r="E38" s="65" t="n">
+        <v>-237.4890071999998</v>
+      </c>
+      <c r="F38" s="65" t="n">
+        <v>-118.4082072000001</v>
+      </c>
+      <c r="G38" s="65" t="n">
+        <v>0.6725928000014392</v>
+      </c>
+      <c r="H38" s="65" t="n">
+        <v>119.7533928000012</v>
+      </c>
+      <c r="I38" s="65" t="n">
+        <v>278.5277928000014</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="66" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" s="65" t="n">
+        <v>-433.8450071999996</v>
+      </c>
+      <c r="D39" s="65" t="n">
+        <v>-314.8290072</v>
+      </c>
+      <c r="E39" s="65" t="n">
+        <v>-195.8130071999985</v>
+      </c>
+      <c r="F39" s="65" t="n">
+        <v>-76.79700719999892</v>
+      </c>
+      <c r="G39" s="65" t="n">
+        <v>42.21899280000071</v>
+      </c>
+      <c r="H39" s="65" t="n">
+        <v>161.2349928000003</v>
+      </c>
+      <c r="I39" s="65" t="n">
+        <v>319.9229928000004</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="66" t="n">
+        <v>7</v>
+      </c>
+      <c r="C40" s="65" t="n">
+        <v>-392.0394072000001</v>
+      </c>
+      <c r="D40" s="65" t="n">
+        <v>-273.0882071999986</v>
+      </c>
+      <c r="E40" s="65" t="n">
+        <v>-154.1370071999991</v>
+      </c>
+      <c r="F40" s="65" t="n">
+        <v>-35.18580719999954</v>
+      </c>
+      <c r="G40" s="65" t="n">
+        <v>83.76539279999997</v>
+      </c>
+      <c r="H40" s="65" t="n">
+        <v>202.7165928000013</v>
+      </c>
+      <c r="I40" s="65" t="n">
+        <v>361.3181928000013</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="66" t="n">
+        <v>8</v>
+      </c>
+      <c r="C41" s="65" t="n">
+        <v>-350.2338072000002</v>
+      </c>
+      <c r="D41" s="65" t="n">
+        <v>-231.347407199999</v>
+      </c>
+      <c r="E41" s="65" t="n">
+        <v>-112.4610071999996</v>
+      </c>
+      <c r="F41" s="65" t="n">
+        <v>6.425392799999827</v>
+      </c>
+      <c r="G41" s="65" t="n">
+        <v>125.3117928000011</v>
+      </c>
+      <c r="H41" s="65" t="n">
+        <v>244.1981928000005</v>
+      </c>
+      <c r="I41" s="65" t="n">
+        <v>402.7133928000003</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>What batteries actually buy you</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>1. Batteries at TODAY'S price (€250/kWh) are roughly break-even in the base case (-€118/GPU/yr) — they're not a magic wand. The spread (grid - curt/eff) only earns over the curtailment days you actually cycle on; below ~200 cycles/yr the fixed cost of the battery outruns the arbitrage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47" ht="32" customHeight="1">
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>2. Where batteries DO pay: deep, frequent curtailment markets. Spain 2030 (-€60 curt, 7h, 240 days) flips to +€504/GPU/yr from adding a battery. The Trifecta best-case adds another €600/yr. The lever is days-of-cycling, more than depth of negative prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49" ht="32" customHeight="1">
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>3. Battery price is the single biggest free variable, with a clear downward trajectory. At €150/kWh (2028 forecast), even the base case turns positive (+€201/GPU/yr). At €400/kWh you actively lose €600/yr. Every €50/kWh of BESS price ≈ €200-400/GPU/yr of EBITDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50"/>
+    <row r="51" ht="32" customHeight="1">
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>4. Round-trip efficiency matters less than you'd think. 88% → 95% only adds ~€50/GPU/yr because most of the cost is amortisation, not energy losses. Don't pay big premiums for high-RTE chemistries here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53" ht="32" customHeight="1">
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>5. The stand-alone arbitrage column (rightmost) shows what the SAME battery would earn with NO GPU at all — just charging cheap and selling expensive. In the base case it's slightly negative; in Spain 2030 it's +€183. Adding GPUs to that BESS adds €321 (€504 - €183) of incremental value over the battery alone. That's the real co-location synergy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55" ht="32" customHeight="1">
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>6. Battery + GPU is a stacked play, not a substitute. You get: AI compute revenue + energy arbitrage + (not modelled here) ancillary services + capacity payments. The base case stack at 2028 prices is meaningfully profitable; today it's marginal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57" ht="32" customHeight="1">
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>7. Batteries do NOT rescue curtailment-only mode. They lower the cost of running 24/7 — which only widens 24/7's lead over Curt-only. The conclusion that 'GPUs should run 24/7' is reinforced, not overturned, by adding storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58"/>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B51:I52"/>
+    <mergeCell ref="B57:I58"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B53:I54"/>
+    <mergeCell ref="B55:I56"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B45:I46"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="D8:I8"/>
+    <mergeCell ref="B49:I50"/>
+    <mergeCell ref="B47:I48"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G14:G20">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25:H30">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C36:I41">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>